<commit_message>
read connection names and node names for mfn connections as well
</commit_message>
<xml_diff>
--- a/tests/formats/mfn_excel/MFN_example_int.xlsx
+++ b/tests/formats/mfn_excel/MFN_example_int.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\en986\Documents\Projects\Alltours\generalized_agv_path_finding\tests\formats\mfn_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B34EE409-E061-431E-9BFA-1DFC709A8E56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90B58AE5-00BB-4648-BF5B-37F63C0296F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30612" yWindow="228" windowWidth="30936" windowHeight="16776" activeTab="1" xr2:uid="{B8DE84FF-B3E8-4D87-8A95-BDBF8C6662ED}"/>
+    <workbookView xWindow="30612" yWindow="228" windowWidth="30936" windowHeight="16776" activeTab="2" xr2:uid="{B8DE84FF-B3E8-4D87-8A95-BDBF8C6662ED}"/>
   </bookViews>
   <sheets>
     <sheet name="NetworkNodes" sheetId="3" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="24">
   <si>
     <t>cal_trans_duration_seconds</t>
   </si>
@@ -48,12 +48,6 @@
   </si>
   <si>
     <t>name</t>
-  </si>
-  <si>
-    <t>1-E1</t>
-  </si>
-  <si>
-    <t>1-E0</t>
   </si>
   <si>
     <t>z_meter</t>
@@ -517,16 +511,16 @@
         <v>4</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -534,7 +528,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C2">
         <v>1.5</v>
@@ -551,7 +545,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C3">
         <v>2.2999999999999998</v>
@@ -568,7 +562,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C4">
         <v>3</v>
@@ -585,7 +579,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C5">
         <v>1.5</v>
@@ -626,7 +620,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>1</v>
@@ -634,7 +628,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -643,15 +637,15 @@
         <v>2</v>
       </c>
       <c r="D2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B3">
         <v>2</v>
@@ -660,15 +654,15 @@
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B4">
         <v>2</v>
@@ -677,15 +671,15 @@
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B5">
         <v>3</v>
@@ -694,10 +688,10 @@
         <v>2</v>
       </c>
       <c r="D5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -730,13 +724,13 @@
         <v>3</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>0</v>
@@ -747,48 +741,48 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B2" t="s">
-        <v>6</v>
+        <v>21</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D2" t="s">
-        <v>5</v>
+        <v>17</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F2" s="6">
         <v>90</v>
       </c>
       <c r="G2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
+        <v>22</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D3" t="s">
-        <v>6</v>
+        <v>18</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
       </c>
       <c r="E3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F3" s="6">
         <v>90</v>
       </c>
       <c r="G3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -809,15 +803,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B2">
         <v>0.5</v>
@@ -825,7 +819,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B3">
         <v>0.4</v>

</xml_diff>